<commit_message>
added parsing to LeiloesJa and MonizDeAragao
</commit_message>
<xml_diff>
--- a/leiloeiros_associados.xlsx
+++ b/leiloeiros_associados.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="177">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -683,7 +683,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -726,6 +726,10 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1169,6 +1173,9 @@
       <c r="F8" s="4" t="s">
         <v>37</v>
       </c>
+      <c r="G8" s="11" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="n">
@@ -1189,6 +1196,9 @@
       <c r="F9" s="7" t="s">
         <v>41</v>
       </c>
+      <c r="G9" s="11" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
@@ -1208,6 +1218,9 @@
       </c>
       <c r="F10" s="4" t="s">
         <v>45</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1229,6 +1242,9 @@
       <c r="F11" s="7" t="s">
         <v>49</v>
       </c>
+      <c r="G11" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
@@ -1249,6 +1265,9 @@
       <c r="F12" s="4" t="s">
         <v>53</v>
       </c>
+      <c r="G12" s="11" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="n">
@@ -1269,6 +1288,9 @@
       <c r="F13" s="7" t="s">
         <v>57</v>
       </c>
+      <c r="G13" s="11" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
@@ -1289,6 +1311,9 @@
       <c r="F14" s="4" t="s">
         <v>61</v>
       </c>
+      <c r="G14" s="11" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="n">
@@ -1309,6 +1334,9 @@
       <c r="F15" s="7" t="s">
         <v>65</v>
       </c>
+      <c r="G15" s="11" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="n">
@@ -1328,6 +1356,9 @@
       </c>
       <c r="F16" s="4" t="s">
         <v>69</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
added PauloBotelhoParser and Navigator
</commit_message>
<xml_diff>
--- a/leiloeiros_associados.xlsx
+++ b/leiloeiros_associados.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="178">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -389,6 +389,9 @@
   </si>
   <si>
     <t xml:space="preserve">(21) 3795-2161 / (21) 99988-3967</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OK</t>
   </si>
   <si>
     <t xml:space="preserve">Mauro Marcello Da Costa Machado</t>
@@ -560,7 +563,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -612,13 +615,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <u val="single"/>
-      <sz val="10"/>
-      <color rgb="FF0563C1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -690,7 +686,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -737,10 +733,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1391,7 +1383,7 @@
       <c r="F17" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="G17" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1414,7 +1406,7 @@
       <c r="F18" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1437,7 +1429,7 @@
       <c r="F19" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G19" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1460,7 +1452,7 @@
       <c r="F20" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1483,7 +1475,7 @@
       <c r="F21" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="G21" s="3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1506,7 +1498,7 @@
       <c r="F22" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1549,7 +1541,7 @@
       <c r="F24" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1592,7 +1584,7 @@
       <c r="F26" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="G26" s="3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1615,7 +1607,7 @@
       <c r="F27" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="G27" s="11" t="s">
+      <c r="G27" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1626,7 +1618,7 @@
       <c r="B28" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="C28" s="5" t="s">
         <v>116</v>
       </c>
       <c r="D28" s="4" t="s">
@@ -1658,25 +1650,31 @@
       <c r="F29" s="7" t="s">
         <v>122</v>
       </c>
+      <c r="G29" s="11" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1684,19 +1682,22 @@
         <v>30</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>9</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1704,19 +1705,22 @@
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
+      </c>
+      <c r="G32" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1724,19 +1728,19 @@
         <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>9</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1744,19 +1748,19 @@
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1764,19 +1768,19 @@
         <v>34</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>9</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1784,19 +1788,19 @@
         <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1804,16 +1808,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>23</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>61</v>
@@ -1824,19 +1828,19 @@
         <v>37</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1844,19 +1848,19 @@
         <v>38</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D39" s="7" t="s">
         <v>9</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1864,19 +1868,19 @@
         <v>39</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1884,16 +1888,16 @@
         <v>40</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D41" s="7" t="s">
         <v>23</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F41" s="7" t="s">
         <v>25</v>
@@ -1904,19 +1908,19 @@
         <v>41</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1924,19 +1928,19 @@
         <v>42</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D43" s="7" t="s">
         <v>9</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
added RodrigoCostaParser and Navigator
</commit_message>
<xml_diff>
--- a/leiloeiros_associados.xlsx
+++ b/leiloeiros_associados.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="178">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -1650,7 +1650,7 @@
       <c r="F29" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="G29" s="11" t="s">
+      <c r="G29" s="3" t="s">
         <v>123</v>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       <c r="F30" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="G30" s="11" t="s">
+      <c r="G30" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       <c r="F31" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="G31" s="11" t="s">
+      <c r="G31" s="3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1719,7 +1719,7 @@
       <c r="F32" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="G32" s="11" t="s">
+      <c r="G32" s="3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1742,6 +1742,9 @@
       <c r="F33" s="7" t="s">
         <v>139</v>
       </c>
+      <c r="G33" s="11" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="n">
@@ -1762,6 +1765,9 @@
       <c r="F34" s="4" t="s">
         <v>143</v>
       </c>
+      <c r="G34" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="n">
@@ -1781,6 +1787,9 @@
       </c>
       <c r="F35" s="7" t="s">
         <v>147</v>
+      </c>
+      <c r="G35" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>